<commit_message>
Updates for task 1B
</commit_message>
<xml_diff>
--- a/Task 1a/Task 1a.xlsx
+++ b/Task 1a/Task 1a.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15735" yWindow="3270" windowWidth="20520" windowHeight="17100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2730" yWindow="2730" windowWidth="17775" windowHeight="17100" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Student" sheetId="1" state="visible" r:id="rId1"/>
@@ -19,12 +19,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +56,12 @@
       <sz val="14"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -82,7 +89,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -175,34 +182,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -228,21 +213,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -265,43 +249,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -325,6 +329,9 @@
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="168" formatCode="0.00000"/>
+    </dxf>
+    <dxf>
       <font>
         <name val="Calibri"/>
         <family val="2"/>
@@ -341,16 +348,13 @@
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <numFmt numFmtId="168" formatCode="0.00000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <numFmt numFmtId="168" formatCode="0.00000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <numFmt numFmtId="168" formatCode="0.00000"/>
     </dxf>
     <dxf>
       <protection locked="0" hidden="0"/>
@@ -605,7 +609,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
@@ -649,19 +653,19 @@
                   <v>0</v>
                 </pt>
                 <pt idx="1">
-                  <v>0.02399999999999999</v>
+                  <v>0.2225</v>
                 </pt>
                 <pt idx="2">
-                  <v>0.06749999999999999</v>
+                  <v>0.4239999999999999</v>
                 </pt>
                 <pt idx="3">
-                  <v>1.0405</v>
+                  <v>1.0485</v>
                 </pt>
                 <pt idx="4">
-                  <v>1.6185</v>
+                  <v>1.6915</v>
                 </pt>
                 <pt idx="5">
-                  <v>1.8175</v>
+                  <v>2.15</v>
                 </pt>
               </numCache>
             </numRef>
@@ -735,6 +739,29 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </txPr>
         </title>
         <numFmt formatCode="0.0" sourceLinked="1"/>
         <majorTickMark val="out"/>
@@ -765,7 +792,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -843,6 +870,29 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-AU"/>
+            </a:p>
+          </txPr>
         </title>
         <numFmt formatCode="0.000" sourceLinked="1"/>
         <majorTickMark val="out"/>
@@ -873,7 +923,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -945,8 +995,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:M6" headerRowCount="1" totalsRowShown="0" headerRowDxfId="12">
-  <autoFilter ref="A1:M6"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:M4" headerRowCount="1" totalsRowShown="0" headerRowDxfId="12">
+  <autoFilter ref="A1:M4"/>
   <tableColumns count="13">
     <tableColumn id="1" name="Student Number" dataDxfId="11"/>
     <tableColumn id="2" name="Target" dataDxfId="10"/>
@@ -966,14 +1016,14 @@
     <tableColumn id="10" name="V 3" dataDxfId="3">
       <calculatedColumnFormula>IF(ISNUMBER(G2),G2/$D2,NA())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" name="V mean" dataDxfId="2">
+    <tableColumn id="11" name="V mean" dataDxfId="1">
       <calculatedColumnFormula>_xlfn.AGGREGATE(1,6,H2:J2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" name="Rel Error" dataDxfId="1" dataCellStyle="Percent">
+    <tableColumn id="12" name="Rel Error" dataDxfId="2" dataCellStyle="Percent">
       <calculatedColumnFormula>ABS(B2-K2)/B2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="13" name="Rel Precision" dataDxfId="0" dataCellStyle="Percent">
-      <calculatedColumnFormula>ABS(MAX(H2:J2)-MIN(H2:J2))/B2</calculatedColumnFormula>
+      <calculatedColumnFormula>ABS(MAX(H2:J2)-MIN(H2:J2))/K2</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1247,46 +1297,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15.85546875" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
-    <col width="13.85546875" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
-    <col width="15.42578125" bestFit="1" customWidth="1" style="41" min="3" max="3"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" style="41" min="4" max="4"/>
-    <col width="9.140625" customWidth="1" style="32" min="19" max="20"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="E1" s="37" t="inlineStr">
+      <c r="E1" s="34" t="inlineStr">
         <is>
           <t>Experimental Data</t>
         </is>
       </c>
-      <c r="F1" s="42" t="n"/>
-      <c r="G1" s="42" t="n"/>
-      <c r="H1" s="43" t="n"/>
-      <c r="I1" s="37" t="inlineStr">
+      <c r="I1" s="34" t="inlineStr">
         <is>
           <t>Data Analysis</t>
         </is>
       </c>
-      <c r="J1" s="42" t="n"/>
-      <c r="K1" s="42" t="n"/>
-      <c r="L1" s="43" t="n"/>
-      <c r="M1" s="37" t="inlineStr">
+      <c r="M1" s="34" t="inlineStr">
         <is>
           <t>Lab Exercises</t>
         </is>
       </c>
-      <c r="N1" s="42" t="n"/>
-      <c r="O1" s="43" t="n"/>
-      <c r="P1" s="37" t="inlineStr">
+      <c r="P1" s="34" t="inlineStr">
         <is>
           <t>References</t>
         </is>
       </c>
-      <c r="Q1" s="43" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1299,77 +1339,77 @@
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C2" s="39" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Partner Number</t>
         </is>
       </c>
-      <c r="D2" s="39" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Partner Name</t>
         </is>
       </c>
-      <c r="E2" s="39" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Tbl 1 2.5</t>
         </is>
       </c>
-      <c r="F2" s="39" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Glc dp 0.5</t>
         </is>
       </c>
-      <c r="G2" s="39" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Part C 2</t>
         </is>
       </c>
-      <c r="H2" s="39" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Part D 1</t>
         </is>
       </c>
-      <c r="I2" s="39" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Q1 0.5</t>
         </is>
       </c>
-      <c r="J2" s="39" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Q2 0.5</t>
         </is>
       </c>
-      <c r="K2" s="39" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Q3 0.5</t>
         </is>
       </c>
-      <c r="L2" s="39" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Q4 0.5</t>
         </is>
       </c>
-      <c r="M2" s="39" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>LabEx1 2</t>
         </is>
       </c>
-      <c r="N2" s="39" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>LabEx2 2</t>
         </is>
       </c>
-      <c r="O2" s="39" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>LabEx3 2</t>
         </is>
       </c>
-      <c r="P2" s="39" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>LitSel 1</t>
         </is>
       </c>
-      <c r="Q2" s="39" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>QualRef 1</t>
         </is>
@@ -1379,136 +1419,10 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="S2" s="32" t="inlineStr">
-        <is>
-          <t>Out of 10</t>
-        </is>
-      </c>
-      <c r="T2" s="32" t="inlineStr">
-        <is>
-          <t>Out of 5</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1234567</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Full Marks</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M3" t="n">
-        <v>2</v>
-      </c>
-      <c r="N3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O3" t="n">
-        <v>2</v>
-      </c>
-      <c r="P3" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>1</v>
-      </c>
       <c r="R3">
         <f>SUM(E3:Q3)</f>
-        <v/>
-      </c>
-      <c r="S3" s="32">
-        <f>R3/2</f>
-        <v/>
-      </c>
-      <c r="T3" s="32">
-        <f>R3/4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>1184207</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Hamish Aldous</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="L4" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N4" t="n">
-        <v>2</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="R4">
-        <f>SUM(E4:Q4)</f>
-        <v/>
-      </c>
-      <c r="S4" s="32">
-        <f>R4/2</f>
-        <v/>
-      </c>
-      <c r="T4" s="32">
-        <f>R4/4</f>
         <v/>
       </c>
     </row>
@@ -1532,30 +1446,31 @@
   <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17.85546875" customWidth="1" style="33" min="1" max="1"/>
-    <col width="12" customWidth="1" style="34" min="2" max="2"/>
-    <col width="9.140625" customWidth="1" style="33" min="3" max="3"/>
-    <col width="9.85546875" customWidth="1" style="41" min="4" max="4"/>
-    <col width="9.140625" customWidth="1" style="33" min="5" max="7"/>
-    <col width="9.140625" customWidth="1" style="9" min="8" max="10"/>
-    <col width="9.85546875" customWidth="1" style="9" min="11" max="11"/>
-    <col width="10.7109375" customWidth="1" style="10" min="12" max="12"/>
-    <col width="14.5703125" customWidth="1" style="10" min="13" max="13"/>
-    <col width="9.85546875" customWidth="1" style="41" min="18" max="18"/>
+    <col width="17.85546875" customWidth="1" style="32" min="1" max="1"/>
+    <col width="12" customWidth="1" style="36" min="2" max="2"/>
+    <col width="9.140625" customWidth="1" style="32" min="3" max="3"/>
+    <col width="9.85546875" customWidth="1" min="4" max="4"/>
+    <col width="9.140625" customWidth="1" style="32" min="5" max="7"/>
+    <col width="9.5703125" bestFit="1" customWidth="1" style="37" min="8" max="8"/>
+    <col width="9.28515625" bestFit="1" customWidth="1" style="37" min="9" max="10"/>
+    <col width="9.85546875" customWidth="1" style="37" min="11" max="11"/>
+    <col width="10.7109375" customWidth="1" style="38" min="12" max="12"/>
+    <col width="14.5703125" customWidth="1" style="38" min="13" max="13"/>
+    <col width="9.85546875" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="33" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>Student Number</t>
         </is>
       </c>
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="36" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C1" s="33" t="inlineStr">
+      <c r="C1" s="32" t="inlineStr">
         <is>
           <t>Temp</t>
         </is>
@@ -1565,47 +1480,47 @@
           <t>Density</t>
         </is>
       </c>
-      <c r="E1" s="33" t="inlineStr">
+      <c r="E1" s="32" t="inlineStr">
         <is>
           <t>Mass 1</t>
         </is>
       </c>
-      <c r="F1" s="33" t="inlineStr">
+      <c r="F1" s="32" t="inlineStr">
         <is>
           <t>Mass 2</t>
         </is>
       </c>
-      <c r="G1" s="33" t="inlineStr">
+      <c r="G1" s="32" t="inlineStr">
         <is>
           <t>Mass 3</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="37" t="inlineStr">
         <is>
           <t>V 1</t>
         </is>
       </c>
-      <c r="I1" s="9" t="inlineStr">
+      <c r="I1" s="37" t="inlineStr">
         <is>
           <t>V 2</t>
         </is>
       </c>
-      <c r="J1" s="9" t="inlineStr">
+      <c r="J1" s="37" t="inlineStr">
         <is>
           <t>V 3</t>
         </is>
       </c>
-      <c r="K1" s="9" t="inlineStr">
+      <c r="K1" s="37" t="inlineStr">
         <is>
           <t>V mean</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="38" t="inlineStr">
         <is>
           <t>Rel Error</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="38" t="inlineStr">
         <is>
           <t>Rel Precision</t>
         </is>
@@ -1622,52 +1537,52 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="32" t="inlineStr">
         <is>
           <t>Test 1000</t>
         </is>
       </c>
-      <c r="B2" s="34" t="n">
+      <c r="B2" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="33" t="n">
+      <c r="C2" s="32" t="n">
         <v>23</v>
       </c>
       <c r="D2">
         <f>VLOOKUP(C2,temp_table[],2)</f>
         <v/>
       </c>
-      <c r="E2" s="33" t="n">
+      <c r="E2" s="32" t="n">
         <v>0.992</v>
       </c>
-      <c r="F2" s="33" t="n">
+      <c r="F2" s="32" t="n">
         <v>0.993</v>
       </c>
-      <c r="G2" s="33" t="n">
+      <c r="G2" s="32" t="n">
         <v>0.993</v>
       </c>
-      <c r="H2" s="9">
+      <c r="H2" s="37">
         <f>IF(ISNUMBER(E2),E2/$D2,NA())</f>
         <v/>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="37">
         <f>IF(ISNUMBER(F2),F2/$D2,NA())</f>
         <v/>
       </c>
-      <c r="J2" s="9">
+      <c r="J2" s="37">
         <f>IF(ISNUMBER(G2),G2/$D2,NA())</f>
         <v/>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="37">
         <f>_xlfn.AGGREGATE(1,6,H2:J2)</f>
         <v/>
       </c>
-      <c r="L2" s="10">
+      <c r="L2" s="38">
         <f>ABS(B2-K2)/B2</f>
         <v/>
       </c>
-      <c r="M2" s="10">
-        <f>ABS(MAX(H2:J2)-MIN(H2:J2))/B2</f>
+      <c r="M2" s="38">
+        <f>ABS(MAX(H2:J2)-MIN(H2:J2))/K2</f>
         <v/>
       </c>
       <c r="Q2" s="3" t="n">
@@ -1678,52 +1593,52 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="33" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>Test 50</t>
         </is>
       </c>
-      <c r="B3" s="34" t="n">
+      <c r="B3" s="36" t="n">
         <v>0.05</v>
       </c>
-      <c r="C3" s="33" t="n">
+      <c r="C3" s="32" t="n">
         <v>23</v>
       </c>
       <c r="D3">
         <f>VLOOKUP(C3,temp_table[],2)</f>
         <v/>
       </c>
-      <c r="E3" s="33" t="n">
+      <c r="E3" s="32" t="n">
         <v>0.051</v>
       </c>
-      <c r="F3" s="33" t="n">
+      <c r="F3" s="32" t="n">
         <v>0.053</v>
       </c>
-      <c r="G3" s="33" t="n">
+      <c r="G3" s="32" t="n">
         <v>0.053</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="37">
         <f>IF(ISNUMBER(E3),E3/$D3,NA())</f>
         <v/>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="37">
         <f>IF(ISNUMBER(F3),F3/$D3,NA())</f>
         <v/>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="37">
         <f>IF(ISNUMBER(G3),G3/$D3,NA())</f>
         <v/>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="37">
         <f>_xlfn.AGGREGATE(1,6,H3:J3)</f>
         <v/>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="38">
         <f>ABS(B3-K3)/B3</f>
         <v/>
       </c>
-      <c r="M3" s="10">
-        <f>ABS(MAX(H3:J3)-MIN(H3:J3))/B3</f>
+      <c r="M3" s="38">
+        <f>ABS(MAX(H3:J3)-MIN(H3:J3))/K3</f>
         <v/>
       </c>
       <c r="Q3" s="3" t="n">
@@ -1734,46 +1649,46 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="33" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>Lab Exercise 1</t>
         </is>
       </c>
-      <c r="B4" s="34" t="n">
+      <c r="B4" s="36" t="n">
         <v>750</v>
       </c>
-      <c r="C4" s="33" t="n">
+      <c r="C4" s="32" t="n">
         <v>25</v>
       </c>
       <c r="D4">
         <f>VLOOKUP(C4,temp_table[],2)</f>
         <v/>
       </c>
-      <c r="E4" s="33" t="n">
+      <c r="E4" s="32" t="n">
         <v>752</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H4" s="37">
         <f>IF(ISNUMBER(E4),E4/$D4,NA())</f>
         <v/>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="37">
         <f>IF(ISNUMBER(F4),F4/$D4,NA())</f>
         <v/>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="37">
         <f>IF(ISNUMBER(G4),G4/$D4,NA())</f>
         <v/>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="37">
         <f>_xlfn.AGGREGATE(1,6,H4:J4)</f>
         <v/>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="38">
         <f>ABS(B4-K4)/B4</f>
         <v/>
       </c>
-      <c r="M4" s="10">
-        <f>ABS(MAX(H4:J4)-MIN(H4:J4))/B4</f>
+      <c r="M4" s="38">
+        <f>ABS(MAX(H4:J4)-MIN(H4:J4))/K4</f>
         <v/>
       </c>
       <c r="Q4" s="3" t="n">
@@ -1784,52 +1699,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="33" t="n">
-        <v>1184207</v>
-      </c>
-      <c r="B5" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="33" t="n">
-        <v>22</v>
-      </c>
-      <c r="D5">
-        <f>VLOOKUP(C5,temp_table[],2)</f>
-        <v/>
-      </c>
-      <c r="E5" s="33" t="n">
-        <v>1.027</v>
-      </c>
-      <c r="F5" s="33" t="n">
-        <v>1.027</v>
-      </c>
-      <c r="G5" s="33" t="n">
-        <v>1.023</v>
-      </c>
-      <c r="H5" s="9">
-        <f>IF(ISNUMBER(E5),E5/$D5,NA())</f>
-        <v/>
-      </c>
-      <c r="I5" s="9">
-        <f>IF(ISNUMBER(F5),F5/$D5,NA())</f>
-        <v/>
-      </c>
-      <c r="J5" s="9">
-        <f>IF(ISNUMBER(G5),G5/$D5,NA())</f>
-        <v/>
-      </c>
-      <c r="K5" s="9">
-        <f>_xlfn.AGGREGATE(1,6,H5:J5)</f>
-        <v/>
-      </c>
-      <c r="L5" s="10">
-        <f>ABS(B5-K5)/B5</f>
-        <v/>
-      </c>
-      <c r="M5" s="10">
-        <f>ABS(MAX(H5:J5)-MIN(H5:J5))/B5</f>
-        <v/>
-      </c>
       <c r="Q5" s="3" t="n">
         <v>23</v>
       </c>
@@ -1838,52 +1707,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="n">
-        <v>1184207</v>
-      </c>
-      <c r="B6" s="34" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>22</v>
-      </c>
-      <c r="D6">
-        <f>VLOOKUP(C6,temp_table[],2)</f>
-        <v/>
-      </c>
-      <c r="E6" s="33" t="n">
-        <v>0.049</v>
-      </c>
-      <c r="F6" s="33" t="n">
-        <v>0.051</v>
-      </c>
-      <c r="G6" s="33" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H6" s="9">
-        <f>IF(ISNUMBER(E6),E6/$D6,NA())</f>
-        <v/>
-      </c>
-      <c r="I6" s="9">
-        <f>IF(ISNUMBER(F6),F6/$D6,NA())</f>
-        <v/>
-      </c>
-      <c r="J6" s="9">
-        <f>IF(ISNUMBER(G6),G6/$D6,NA())</f>
-        <v/>
-      </c>
-      <c r="K6" s="9">
-        <f>_xlfn.AGGREGATE(1,6,H6:J6)</f>
-        <v/>
-      </c>
-      <c r="L6" s="10">
-        <f>ABS(B6-K6)/B6</f>
-        <v/>
-      </c>
-      <c r="M6" s="10">
-        <f>ABS(MAX(H6:J6)-MIN(H6:J6))/B6</f>
-        <v/>
-      </c>
       <c r="Q6" s="3" t="n">
         <v>24</v>
       </c>
@@ -1917,30 +1740,30 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19.140625" customWidth="1" style="12" min="1" max="1"/>
-    <col width="17.85546875" customWidth="1" style="1" min="2" max="2"/>
-    <col width="15.28515625" customWidth="1" style="1" min="3" max="3"/>
+    <col width="19.140625" customWidth="1" style="39" min="1" max="1"/>
+    <col width="17.85546875" customWidth="1" style="34" min="2" max="2"/>
+    <col width="15.28515625" customWidth="1" style="34" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customFormat="1" customHeight="1" s="11">
-      <c r="A1" s="13" t="inlineStr">
+    <row r="1" ht="30" customFormat="1" customHeight="1" s="10">
+      <c r="A1" s="40" t="inlineStr">
         <is>
           <t>Glucose Standard (mmol/L)</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Vol 10 mmol/L Stock (uL)</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Vol DI Water (uL)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="n">
+      <c r="A2" s="41" t="n">
         <v>0</v>
       </c>
       <c r="B2" s="2">
@@ -1953,7 +1776,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="15" t="n">
+      <c r="A3" s="41" t="n">
         <v>0.1</v>
       </c>
       <c r="B3" s="2">
@@ -1966,7 +1789,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="41" t="n">
         <v>0.2</v>
       </c>
       <c r="B4" s="2">
@@ -1979,7 +1802,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="41" t="n">
         <v>0.5</v>
       </c>
       <c r="B5" s="2">
@@ -1992,7 +1815,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="n">
+      <c r="A6" s="41" t="n">
         <v>0.8</v>
       </c>
       <c r="B6" s="2">
@@ -2005,7 +1828,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="41" t="n">
         <v>1</v>
       </c>
       <c r="B7" s="2">
@@ -2031,104 +1854,104 @@
   <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.28515625" customWidth="1" style="41" min="2" max="2"/>
-    <col width="12.7109375" customWidth="1" style="41" min="3" max="5"/>
-    <col width="13.7109375" customWidth="1" style="41" min="6" max="6"/>
-    <col width="16.28515625" customWidth="1" style="41" min="8" max="8"/>
+    <col width="12.28515625" customWidth="1" min="2" max="2"/>
+    <col width="12.7109375" customWidth="1" min="3" max="5"/>
+    <col width="13.7109375" customWidth="1" min="6" max="6"/>
+    <col width="16.28515625" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" s="41">
-      <c r="A1" s="16" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Practical 1:  Glucose Standard Curve</t>
         </is>
       </c>
-      <c r="B1" s="17" t="n"/>
-      <c r="C1" s="17" t="n"/>
-      <c r="D1" s="17" t="n"/>
-      <c r="E1" s="17" t="n"/>
-      <c r="F1" s="17" t="n"/>
+      <c r="B1" s="16" t="n"/>
+      <c r="C1" s="16" t="n"/>
+      <c r="D1" s="16" t="n"/>
+      <c r="E1" s="16" t="n"/>
+      <c r="F1" s="16" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Enter your absorbance values into the table below.</t>
         </is>
       </c>
-      <c r="B3" s="19" t="n"/>
-      <c r="C3" s="19" t="n"/>
-      <c r="D3" s="19" t="n"/>
-      <c r="E3" s="19" t="n"/>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="B3" s="18" t="n"/>
+      <c r="C3" s="18" t="n"/>
+      <c r="D3" s="18" t="n"/>
+      <c r="E3" s="18" t="n"/>
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>For the trendline, select intercept at 0, equation for the line, and r2 value</t>
         </is>
       </c>
-      <c r="I3" s="19" t="n"/>
-      <c r="J3" s="19" t="n"/>
-      <c r="K3" s="19" t="n"/>
-      <c r="L3" s="19" t="n"/>
-      <c r="M3" s="19" t="n"/>
-      <c r="N3" s="19" t="n"/>
-    </row>
-    <row r="5" ht="57.6" customFormat="1" customHeight="1" s="23">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="I3" s="18" t="n"/>
+      <c r="J3" s="18" t="n"/>
+      <c r="K3" s="18" t="n"/>
+      <c r="L3" s="18" t="n"/>
+      <c r="M3" s="18" t="n"/>
+      <c r="N3" s="18" t="n"/>
+    </row>
+    <row r="5" ht="57.6" customFormat="1" customHeight="1" s="22">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>Tube</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Glucose conc. (mmol/L)</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Duplicate Absorbance 1 (Units)</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Duplicate Absorbance 2 (Units)</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>Mean Absorbance (Units)</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="20" t="inlineStr">
         <is>
           <t>Mean Blank Adjust Absorbance (Units)</t>
         </is>
       </c>
-      <c r="G5" s="22" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>Include</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="42">
         <f>IF(G6="yes",0,NA())</f>
         <v/>
       </c>
-      <c r="C6" s="26" t="n">
-        <v>0.083</v>
-      </c>
-      <c r="D6" s="26" t="n">
-        <v>0.082</v>
-      </c>
-      <c r="E6" s="26">
+      <c r="C6" s="43" t="n">
+        <v>0.117</v>
+      </c>
+      <c r="D6" s="43" t="n">
+        <v>0.099</v>
+      </c>
+      <c r="E6" s="43">
         <f>IF(ISNUMBER(C6),AVERAGE(C6:D6),"")</f>
         <v/>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="43">
         <f>IF(AND(ISNUMBER(E6),ISNUMBER($E$6),G6="yes"),E6-$E$6,NA())</f>
         <v/>
       </c>
@@ -2139,26 +1962,26 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="42">
         <f>IF(G7="yes",0.1,NA())</f>
         <v/>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>0.091</v>
-      </c>
-      <c r="D7" s="26" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="E7" s="26">
+      <c r="C7" s="43" t="n">
+        <v>0.245</v>
+      </c>
+      <c r="D7" s="43" t="n">
+        <v>0.263</v>
+      </c>
+      <c r="E7" s="43">
         <f>IF(ISNUMBER(C7),AVERAGE(C7:D7),"")</f>
         <v/>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="43">
         <f>IF(AND(ISNUMBER(E7),ISNUMBER($E$6),G7="yes"),E7-$E$6,NA())</f>
         <v/>
       </c>
@@ -2169,26 +1992,26 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="42">
         <f>IF(G8="yes",0.2,NA())</f>
         <v/>
       </c>
-      <c r="C8" s="26" t="n">
-        <v>0.149</v>
-      </c>
-      <c r="D8" s="26" t="n">
-        <v>0.151</v>
-      </c>
-      <c r="E8" s="26">
+      <c r="C8" s="43" t="n">
+        <v>0.448</v>
+      </c>
+      <c r="D8" s="43" t="n">
+        <v>0.443</v>
+      </c>
+      <c r="E8" s="43">
         <f>IF(ISNUMBER(C8),AVERAGE(C8:D8),"")</f>
         <v/>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="43">
         <f>IF(AND(ISNUMBER(E8),ISNUMBER($E$6),G8="yes"),E8-$E$6,NA())</f>
         <v/>
       </c>
@@ -2199,26 +2022,26 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="42">
         <f>IF(G9="yes",0.5,NA())</f>
         <v/>
       </c>
-      <c r="C9" s="26" t="n">
-        <v>1.127</v>
-      </c>
-      <c r="D9" s="26" t="n">
-        <v>1.119</v>
-      </c>
-      <c r="E9" s="26">
+      <c r="C9" s="43" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>1.045</v>
+      </c>
+      <c r="E9" s="43">
         <f>IF(ISNUMBER(C9),AVERAGE(C9:D9),"")</f>
         <v/>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="43">
         <f>IF(AND(ISNUMBER(E9),ISNUMBER($E$6),G9="yes"),E9-$E$6,NA())</f>
         <v/>
       </c>
@@ -2229,26 +2052,26 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="42">
         <f>IF(G10="yes",0.8,NA())</f>
         <v/>
       </c>
-      <c r="C10" s="26" t="n">
-        <v>1.649</v>
-      </c>
-      <c r="D10" s="26" t="n">
-        <v>1.753</v>
-      </c>
-      <c r="E10" s="26">
+      <c r="C10" s="43" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D10" s="43" t="n">
+        <v>1.613</v>
+      </c>
+      <c r="E10" s="43">
         <f>IF(ISNUMBER(C10),AVERAGE(C10:D10),"")</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="43">
         <f>IF(AND(ISNUMBER(E10),ISNUMBER($E$6),G10="yes"),E10-$E$6,NA())</f>
         <v/>
       </c>
@@ -2259,26 +2082,26 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="42">
         <f>IF(G11="yes",1,NA())</f>
         <v/>
       </c>
-      <c r="C11" s="26" t="n">
-        <v>1.717</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>2.083</v>
-      </c>
-      <c r="E11" s="26">
+      <c r="C11" s="43" t="n">
+        <v>2.013</v>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>2.036</v>
+      </c>
+      <c r="E11" s="43">
         <f>IF(ISNUMBER(C11),AVERAGE(C11:D11),"")</f>
         <v/>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="43">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($E$6),G11="yes"),E11-$E$6,NA())</f>
         <v/>
       </c>
@@ -2289,47 +2112,47 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="n"/>
-      <c r="B12" s="27" t="n"/>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
+      <c r="A12" s="26" t="n"/>
+      <c r="B12" s="26" t="n"/>
+      <c r="C12" s="44" t="n"/>
+      <c r="D12" s="44" t="n"/>
+      <c r="E12" s="44" t="n"/>
+      <c r="F12" s="44" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="n"/>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="30" t="n"/>
-      <c r="F13" s="30" t="n"/>
+      <c r="A13" s="28" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="45" t="n"/>
+      <c r="D13" s="45" t="n"/>
+      <c r="E13" s="45" t="n"/>
+      <c r="F13" s="45" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="29" t="n"/>
-      <c r="B14" s="29" t="n"/>
-      <c r="C14" s="30" t="n"/>
-      <c r="D14" s="30" t="n"/>
-      <c r="E14" s="30" t="n"/>
-      <c r="F14" s="30" t="n"/>
+      <c r="A14" s="28" t="n"/>
+      <c r="B14" s="28" t="n"/>
+      <c r="C14" s="45" t="n"/>
+      <c r="D14" s="45" t="n"/>
+      <c r="E14" s="45" t="n"/>
+      <c r="F14" s="45" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="n"/>
-      <c r="B15" s="29" t="n"/>
-      <c r="C15" s="30" t="n"/>
-      <c r="D15" s="30" t="n"/>
-      <c r="E15" s="30" t="n"/>
-      <c r="F15" s="30" t="n"/>
+      <c r="A15" s="28" t="n"/>
+      <c r="B15" s="28" t="n"/>
+      <c r="C15" s="45" t="n"/>
+      <c r="D15" s="45" t="n"/>
+      <c r="E15" s="45" t="n"/>
+      <c r="F15" s="45" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="n"/>
-      <c r="B16" s="29" t="n"/>
-      <c r="C16" s="30" t="n"/>
-      <c r="D16" s="30" t="n"/>
-      <c r="E16" s="30" t="n"/>
-      <c r="F16" s="30" t="n"/>
+      <c r="A16" s="28" t="n"/>
+      <c r="B16" s="28" t="n"/>
+      <c r="C16" s="45" t="n"/>
+      <c r="D16" s="45" t="n"/>
+      <c r="E16" s="45" t="n"/>
+      <c r="F16" s="45" t="n"/>
     </row>
     <row r="17">
-      <c r="H17" s="31" t="inlineStr">
+      <c r="H17" s="30" t="inlineStr">
         <is>
           <t>Data Analysis 4</t>
         </is>
@@ -2365,7 +2188,7 @@
           <t>Glucose (mmol/L)</t>
         </is>
       </c>
-      <c r="I20" s="32">
+      <c r="I20" s="46">
         <f>5*I19/I18</f>
         <v/>
       </c>
@@ -2388,274 +2211,214 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13.7109375" bestFit="1" customWidth="1" style="41" min="1" max="1"/>
-    <col width="12" bestFit="1" customWidth="1" style="41" min="2" max="2"/>
+    <col width="13.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Lab Exercise 1</t>
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Lab Exercise 2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Temp</t>
+          <t>Lactose MW</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>342.3</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>g/mol</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>V1 Reqd</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>DI Water</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>C2 Actual</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>DI Water</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Density</t>
-        </is>
-      </c>
-      <c r="B3">
-        <f>VLOOKUP(B2,temp_table[],2)</f>
+          <t>Mass</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.712</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3">
+        <f>H3*I3/F3</f>
+        <v/>
+      </c>
+      <c r="H3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J3">
+        <f>I3-G3</f>
+        <v/>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>50</v>
+      </c>
+      <c r="N3" t="n">
+        <v>32</v>
+      </c>
+      <c r="O3">
+        <f>M3*N3/P3</f>
+        <v/>
+      </c>
+      <c r="P3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Q3">
+        <f>P3-N3</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mass</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>752</v>
+        <v>100</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4">
+        <f>H4*I4/F4</f>
+        <v/>
+      </c>
+      <c r="H4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J4">
+        <f>I4-G4</f>
+        <v/>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>50</v>
+      </c>
+      <c r="N4" t="n">
+        <v>8</v>
+      </c>
+      <c r="O4">
+        <f>M4*N4/P4</f>
+        <v/>
+      </c>
+      <c r="P4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="Q4">
+        <f>P4-N4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Volume</t>
-        </is>
-      </c>
-      <c r="B5" s="35">
-        <f>B4/B3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Relative error</t>
-        </is>
-      </c>
-      <c r="B6" s="36">
-        <f>ABS(B5-750)/750</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="31" t="inlineStr">
-        <is>
-          <t>Lab Exercise 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Lactose MW</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>342.3</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>g/mol</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>V1 Reqd</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>DI Water</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>V1</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>C2 Actual</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>DI Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mass</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1.712</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>g</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
-        <v>50</v>
-      </c>
-      <c r="G10">
-        <f>H10*I10/F10</f>
-        <v/>
-      </c>
-      <c r="H10" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J10">
-        <f>I10-G10</f>
-        <v/>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="M10" t="n">
-        <v>50</v>
-      </c>
-      <c r="N10" t="n">
-        <v>32</v>
-      </c>
-      <c r="O10">
-        <f>M10*N10/P10</f>
-        <v/>
-      </c>
-      <c r="P10" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Q10">
-        <f>P10-N10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Volume</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>100</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>mL</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>50</v>
-      </c>
-      <c r="G11">
-        <f>H11*I11/F11</f>
-        <v/>
-      </c>
-      <c r="H11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="I11" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J11">
-        <f>I11-G11</f>
-        <v/>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="M11" t="n">
-        <v>50</v>
-      </c>
-      <c r="N11" t="n">
-        <v>8</v>
-      </c>
-      <c r="O11">
-        <f>M11*N11/P11</f>
-        <v/>
-      </c>
-      <c r="P11" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Q11">
-        <f>P11-N11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
           <t>Concentration</t>
         </is>
       </c>
-      <c r="B12">
-        <f>1000*B10/B9/(B11/1000)</f>
-        <v/>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B5">
+        <f>1000*B3/B2/(B4/1000)</f>
+        <v/>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>mmol/L</t>
         </is>

</xml_diff>